<commit_message>
Adding the changes done to stepfile and feature file related to excel driven data
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Exceldata.xlsx
+++ b/src/test/resources/testData/Exceldata.xlsx
@@ -3,38 +3,29 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{802D4A1A-BB8D-4D48-82FF-144A15DF2BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5687DE57-7F32-4F78-A814-DD8CF0BBFD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{5BEF246F-8384-44F0-BBA3-617C41ABE8CE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{5BEF246F-8384-44F0-BBA3-617C41ABE8CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Redirect" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet5" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:L15"/>
+  <oleSize ref="A1:L9"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
   <si>
     <t>Key</t>
   </si>
@@ -127,6 +118,9 @@
   </si>
   <si>
     <t>Sneha_Support</t>
+  </si>
+  <si>
+    <t>]</t>
   </si>
 </sst>
 </file>
@@ -646,13 +640,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C791023-C9F6-417C-A72A-B4937217DCFD}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="22.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -660,7 +654,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>14</v>
       </c>
@@ -668,15 +662,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -684,7 +681,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
@@ -692,7 +689,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Added Properties File and Excel for HttpMethod
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Exceldata.xlsx
+++ b/src/test/resources/testData/Exceldata.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{35630FF5-DB35-419E-BE3C-F4F8FCCAA355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
-    <sheet r:id="rId2" sheetId="2" name="Sheet2"/>
-    <sheet r:id="rId3" sheetId="3" name="Sheet3"/>
-    <sheet r:id="rId4" sheetId="4" name="Sheet4"/>
-    <sheet r:id="rId5" sheetId="5" name="Sheet5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:Q14"/>
 </workbook>
 </file>
 
@@ -122,8 +124,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -180,62 +181,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -246,10 +244,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -287,71 +285,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -379,7 +377,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -402,11 +400,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -415,13 +413,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -431,7 +429,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -440,7 +438,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -449,7 +447,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -457,10 +455,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -525,18 +523,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -544,7 +542,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -552,11 +550,11 @@
         <v>204</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
-      <c r="B3" s="15"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="B3" s="13"/>
+    </row>
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="4"/>
     </row>
@@ -566,46 +564,46 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>101</v>
       </c>
     </row>
@@ -615,72 +613,70 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5546875" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="11">
         <v>9</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <v>7</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="11">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>5</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <v>3</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="11">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>3</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <v>1</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="11">
         <v>5</v>
       </c>
     </row>
@@ -690,18 +686,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="22.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -709,7 +705,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -717,7 +713,7 @@
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>14</v>
       </c>
@@ -725,7 +721,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -733,7 +729,7 @@
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="5" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -741,7 +737,7 @@
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="6" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>20</v>
       </c>
@@ -755,19 +751,19 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="7" width="15.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="17.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -778,7 +774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="2" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>994</v>
       </c>
@@ -789,7 +785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="3" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>105</v>
       </c>
@@ -800,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="4" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>202</v>
       </c>
@@ -811,7 +807,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="5" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>550</v>
       </c>
@@ -822,7 +818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="6" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>888</v>
       </c>

</xml_diff>

<commit_message>
Authorization added Redirect Module
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Exceldata.xlsx
+++ b/src/test/resources/testData/Exceldata.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{3831230D-18B6-4AE7-9974-4688A1300155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D4AA2DDD-5554-4A46-88FB-F2D53968495B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="13104" windowHeight="12336" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,17 +16,6 @@
   </sheets>
   <calcPr calcId="0"/>
   <oleSize ref="A1:O6"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -698,10 +687,10 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13.5546875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="22.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="37.5546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="1" spans="1:2" s="1" customFormat="1">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -709,7 +698,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="2" spans="1:2" s="1" customFormat="1">
       <c r="A2" s="8" t="s">
         <v>14</v>
       </c>
@@ -717,7 +706,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="3" spans="1:2" s="1" customFormat="1">
       <c r="A3" s="8" t="s">
         <v>15</v>
       </c>
@@ -725,7 +714,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="4" spans="1:2" s="1" customFormat="1">
       <c r="A4" s="8" t="s">
         <v>19</v>
       </c>
@@ -733,7 +722,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="5" spans="1:2" s="1" customFormat="1">
       <c r="A5" s="8" t="s">
         <v>21</v>
       </c>
@@ -741,7 +730,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1">
+    <row r="6" spans="1:2" s="1" customFormat="1" ht="28.8">
       <c r="A6" s="8" t="s">
         <v>23</v>
       </c>
@@ -751,6 +740,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Added Authorization for the http methods module
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Exceldata.xlsx
+++ b/src/test/resources/testData/Exceldata.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{CEE00EC8-D5BB-4140-A428-F829E231A4E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
-    <sheet r:id="rId2" sheetId="2" name="Sheet2"/>
-    <sheet r:id="rId3" sheetId="3" name="Sheet3"/>
-    <sheet r:id="rId4" sheetId="4" name="Sheet4"/>
-    <sheet r:id="rId5" sheetId="5" name="Sheet5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1:P5"/>
 </workbook>
 </file>
 
@@ -122,8 +124,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -180,62 +181,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -246,10 +244,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -287,71 +285,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -379,7 +377,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -402,11 +400,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -415,13 +413,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -431,7 +429,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -440,7 +438,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -449,7 +447,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -457,10 +455,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -525,18 +523,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -544,7 +542,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -552,11 +550,11 @@
         <v>204</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5"/>
-      <c r="B3" s="15"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5" customFormat="1" s="1">
+      <c r="B3" s="13"/>
+    </row>
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="4"/>
     </row>
@@ -566,46 +564,46 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>101</v>
       </c>
     </row>
@@ -615,72 +613,70 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="13.5546875" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="11">
         <v>9</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <v>7</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="11">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>5</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <v>3</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="11">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>3</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <v>1</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="11">
         <v>5</v>
       </c>
     </row>
@@ -690,18 +686,18 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="22.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" style="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -709,7 +705,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -717,7 +713,7 @@
         <v>13</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>14</v>
       </c>
@@ -725,7 +721,7 @@
         <v>15</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -733,7 +729,7 @@
         <v>17</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="5" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -741,7 +737,7 @@
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="6" spans="1:2" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>20</v>
       </c>
@@ -755,19 +751,19 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="7" width="15.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="17.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="15.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5" customFormat="1" s="1">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -778,7 +774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="2" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>994</v>
       </c>
@@ -789,7 +785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="3" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>105</v>
       </c>
@@ -800,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="4" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>202</v>
       </c>
@@ -811,7 +807,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="5" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>550</v>
       </c>
@@ -822,7 +818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="6" spans="1:3" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>888</v>
       </c>

</xml_diff>

<commit_message>
Updated Feature file and step definition file
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/Exceldata.xlsx
+++ b/src/test/resources/testData/Exceldata.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{88BEC719-4F5D-4407-BD2B-6CC382A112AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FA13B54A-576A-4DEE-B037-C4CEA27F3A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
     <sheet name="Sheet5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:Q18"/>
+  <oleSize ref="A1:S11"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>

</xml_diff>